<commit_message>
Say where the rules come from, so Rules and Rules v2 read as different things
Both are plain code with no model in the path. Rules runs on the rules the
team already knew; Rules v2 runs on every rule written down during the agent
build. The cards, the legend under every column, the PDF and the workbook now
say so, and one note under the cards says what to do if that spec work has
not been done.

Co-Authored-By: Claude Opus 5 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/public/downloads/agent-run-cost-model.xlsx
+++ b/public/downloads/agent-run-cost-model.xlsx
@@ -565,7 +565,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A61"/>
+  <dimension ref="A1:A62"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="110" customWidth="1" min="1" max="1"/>
@@ -606,10 +606,10 @@
         </is>
       </c>
     </row>
-    <row r="7" ht="30" customHeight="1">
+    <row r="7" ht="45" customHeight="1">
       <c r="A7" s="5" t="inlineStr">
         <is>
-          <t>Four options are compared side by side over one period: a rules workflow, the same rules rebuilt on a written spec, a model that drafts while a person approves, and a full agent with tools.</t>
+          <t>Four options are compared side by side over one period: a rules workflow as first written, the same workflow rebuilt on the decision rules the agent build forced the team to write down, a model that drafts while a person approves, and a full agent with tools.</t>
         </is>
       </c>
     </row>
@@ -718,17 +718,17 @@
         </is>
       </c>
     </row>
-    <row r="26" ht="15" customHeight="1">
+    <row r="26" ht="45" customHeight="1">
       <c r="A26" s="5" t="inlineStr">
         <is>
-          <t>Rules workflow: Plain code that follows fixed rules. No model anywhere in the path.</t>
-        </is>
-      </c>
-    </row>
-    <row r="27" ht="30" customHeight="1">
+          <t>Rules workflow, as first written: Plain code that follows fixed rules, written from what the team already knew. No model anywhere in the path. It handles the common cases and declines or escalates the rest, because the rules for the hard cases were never written down.</t>
+        </is>
+      </c>
+    </row>
+    <row r="27" ht="60" customHeight="1">
       <c r="A27" s="5" t="inlineStr">
         <is>
-          <t>Rules v2, on the written spec: The same code, rebuilt on the decision rules the agent build forced the team to write down.</t>
+          <t>Rules v2, rebuilt on the written spec: The same kind of plain code, rebuilt after the agent was built. Building the agent forced the team to write every decision rule down. Code rebuilt on that written spec covers more cases and declines fewer, so it costs more to build and less to run. Still no model in the path.</t>
         </is>
       </c>
     </row>
@@ -746,183 +746,190 @@
         </is>
       </c>
     </row>
-    <row r="31">
-      <c r="A31" s="4" t="inlineStr">
+    <row r="30" ht="60" customHeight="1">
+      <c r="A30" s="8" t="inlineStr">
+        <is>
+          <t>Rules and Rules v2 are both plain code with no model in the path. The difference is where the rules came from. Rules runs on the rules the team already knew. Rules v2 runs on every rule that got written down while the agent was being built, which is why it handles more cases and costs more to build. If you have not done that spec work, set the Rules v2 column equal to Rules, or leave it blank.</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="4" t="inlineStr">
         <is>
           <t>Rules for using it in a budget conversation</t>
         </is>
       </c>
     </row>
-    <row r="32" ht="45" customHeight="1">
-      <c r="A32" s="5" t="inlineStr">
+    <row r="33" ht="45" customHeight="1">
+      <c r="A33" s="5" t="inlineStr">
         <is>
           <t>Fill it from a trial, not from a guess. Escalation share, review minutes and the retry multiplier come from logs of real cases. A demo produces none of them. Nothing here is a benchmark: there is no industry number for your escalation rate.</t>
         </is>
       </c>
     </row>
-    <row r="33" ht="30" customHeight="1">
-      <c r="A33" s="5" t="inlineStr">
+    <row r="34" ht="30" customHeight="1">
+      <c r="A34" s="5" t="inlineStr">
         <is>
           <t>Argue about cost per acceptable outcome, not cost per case. Cost per case rewards a system that quietly declines the hard cases. Cost per acceptable outcome charges it for them.</t>
         </is>
       </c>
     </row>
-    <row r="34" ht="45" customHeight="1">
-      <c r="A34" s="5" t="inlineStr">
+    <row r="35" ht="45" customHeight="1">
+      <c r="A35" s="5" t="inlineStr">
         <is>
           <t>One definition of an acceptable outcome, one reviewer, all four options. The acceptable-outcome rate must come from one written definition, applied to every option by the same person. Otherwise the comparison is theatre.</t>
         </is>
       </c>
     </row>
-    <row r="35" ht="30" customHeight="1">
-      <c r="A35" s="5" t="inlineStr">
+    <row r="36" ht="30" customHeight="1">
+      <c r="A36" s="5" t="inlineStr">
         <is>
           <t>Blank means unknown. Zero means measured. A blank keeps the result off the screen until you know the number. Type a 0 only when you have measured a 0. "This system never retries" is a claim.</t>
         </is>
       </c>
     </row>
-    <row r="36" ht="45" customHeight="1">
-      <c r="A36" s="5" t="inlineStr">
+    <row r="37" ht="45" customHeight="1">
+      <c r="A37" s="5" t="inlineStr">
         <is>
           <t>Change the rows, keep the shape. Add a cost line your workload has and this model does not: data labelling, a vendor licence, a second reviewer for high-value decisions. The shape is the point: build kept apart from run, quality beside cost, and the operating lines visible.</t>
         </is>
       </c>
     </row>
-    <row r="38">
-      <c r="A38" s="4" t="inlineStr">
+    <row r="39">
+      <c r="A39" s="4" t="inlineStr">
         <is>
           <t>How the outcome is read</t>
         </is>
       </c>
     </row>
-    <row r="39" ht="30" customHeight="1">
-      <c r="A39" s="8" t="inlineStr">
+    <row r="40" ht="30" customHeight="1">
+      <c r="A40" s="8" t="inlineStr">
         <is>
           <t>The leading option is the one with the lowest cost per acceptable outcome among the options that save money against the manual baseline over the period. The last row of each model sheet names it.</t>
-        </is>
-      </c>
-    </row>
-    <row r="40" ht="60" customHeight="1">
-      <c r="A40" s="5" t="inlineStr">
-        <is>
-          <t>The full agent earns its keep — The full agent has the lowest cost per acceptable outcome and beats the manual baseline. Before you commit, measure the three lines that drive this number in a trial: escalation share, review minutes and the retry multiplier. If the trial moves any of them, run the model again before the budget conversation.</t>
         </is>
       </c>
     </row>
     <row r="41" ht="60" customHeight="1">
       <c r="A41" s="5" t="inlineStr">
         <is>
-          <t>Draft with a model, approve with a person — The model-assisted draft has the lowest cost per acceptable outcome and beats the manual baseline. Every case still passes a reviewer, so review minutes per case is the line that decides this. Time it on real cases, not on a demo. If review time doubles, check whether the full agent or the rules workflow now leads.</t>
+          <t>The full agent earns its keep — The full agent has the lowest cost per acceptable outcome and beats the manual baseline. Before you commit, measure the three lines that drive this number in a trial: escalation share, review minutes and the retry multiplier. If the trial moves any of them, run the model again before the budget conversation.</t>
         </is>
       </c>
     </row>
     <row r="42" ht="60" customHeight="1">
       <c r="A42" s="5" t="inlineStr">
         <is>
-          <t>The written spec is the asset. Run the code. — The rebuilt rules workflow has the lowest cost per acceptable outcome and beats the manual baseline. The agent build paid for itself by forcing the team to write the decision rules down. Ship the rebuilt rules workflow, and keep the specification under version control like any other code. Revisit the model when volume or the price of a call changes.</t>
+          <t>Draft with a model, approve with a person — The model-assisted draft has the lowest cost per acceptable outcome and beats the manual baseline. Every case still passes a reviewer, so review minutes per case is the line that decides this. Time it on real cases, not on a demo. If review time doubles, check whether the full agent or the rules workflow now leads.</t>
         </is>
       </c>
     </row>
     <row r="43" ht="60" customHeight="1">
       <c r="A43" s="5" t="inlineStr">
         <is>
+          <t>The written spec is the asset. Run the code. — The rebuilt rules workflow has the lowest cost per acceptable outcome and beats the manual baseline. The agent build paid for itself by forcing the team to write the decision rules down. Ship the rebuilt rules workflow, and keep the specification under version control like any other code. Revisit the model when volume or the price of a call changes.</t>
+        </is>
+      </c>
+    </row>
+    <row r="44" ht="60" customHeight="1">
+      <c r="A44" s="5" t="inlineStr">
+        <is>
           <t>The rules workflow wins as it stands — The original rules workflow has the lowest cost per acceptable outcome and beats the manual baseline. No model earns its cost on this workload at these rates. Keep the rules workflow. Check the acceptable-outcome rate first: if the rules workflow declines a lot of cases, its quality line may be the one that is wrong.</t>
         </is>
       </c>
     </row>
-    <row r="44" ht="45" customHeight="1">
-      <c r="A44" s="5" t="inlineStr">
+    <row r="45" ht="45" customHeight="1">
+      <c r="A45" s="5" t="inlineStr">
         <is>
           <t>Nothing here beats doing it by hand — No option saves money against the manual baseline over the period. Either the volume is too low to earn back a build, or a rate needs checking. Do not build for cost. Build only if there is another reason, and write that reason down in the decision record.</t>
         </is>
       </c>
     </row>
-    <row r="46">
-      <c r="A46" s="4" t="inlineStr">
+    <row r="47">
+      <c r="A47" s="4" t="inlineStr">
         <is>
           <t>The nine lines teams leave out</t>
         </is>
       </c>
     </row>
-    <row r="47" ht="45" customHeight="1">
-      <c r="A47" s="5" t="inlineStr">
+    <row r="48" ht="45" customHeight="1">
+      <c r="A48" s="5" t="inlineStr">
         <is>
           <t>retry and failure multiplier · review minutes per reviewed case · engineer minutes per escalation · share of cases declined or abandoned · observability and eval tooling · eval maintenance · model-version re-qualification · prompt and regression testing · incident and on-call load</t>
         </is>
       </c>
     </row>
-    <row r="49">
-      <c r="A49" s="4" t="inlineStr">
+    <row r="50">
+      <c r="A50" s="4" t="inlineStr">
         <is>
           <t>What this model does not price</t>
-        </is>
-      </c>
-    </row>
-    <row r="50" ht="15" customHeight="1">
-      <c r="A50" s="5" t="inlineStr">
-        <is>
-          <t>It assumes steady volume, one workload and stable rates for the whole period.</t>
         </is>
       </c>
     </row>
     <row r="51" ht="15" customHeight="1">
       <c r="A51" s="5" t="inlineStr">
         <is>
+          <t>It assumes steady volume, one workload and stable rates for the whole period.</t>
+        </is>
+      </c>
+    </row>
+    <row r="52" ht="15" customHeight="1">
+      <c r="A52" s="5" t="inlineStr">
+        <is>
           <t>It does not price revenue upside. A system that wins new business is not captured by a cost line.</t>
-        </is>
-      </c>
-    </row>
-    <row r="52" ht="30" customHeight="1">
-      <c r="A52" s="5" t="inlineStr">
-        <is>
-          <t>It does not price the risk of a wrong action that cannot be undone. That belongs in the Agent Authority Review, not in a cell here.</t>
         </is>
       </c>
     </row>
     <row r="53" ht="30" customHeight="1">
       <c r="A53" s="5" t="inlineStr">
         <is>
+          <t>It does not price the risk of a wrong action that cannot be undone. That belongs in the Agent Authority Review, not in a cell here.</t>
+        </is>
+      </c>
+    </row>
+    <row r="54" ht="30" customHeight="1">
+      <c r="A54" s="5" t="inlineStr">
+        <is>
           <t>It does not price the option value of the capability you build. If that is the argument, write it in the decision record in words, not as a number in this sheet.</t>
         </is>
       </c>
     </row>
-    <row r="55">
-      <c r="A55" s="9" t="inlineStr">
+    <row r="56">
+      <c r="A56" s="9" t="inlineStr">
         <is>
           <t>Join the cohort</t>
-        </is>
-      </c>
-    </row>
-    <row r="56" ht="15" customHeight="1">
-      <c r="A56" s="10" t="inlineStr">
-        <is>
-          <t>The Living Craft is a 6-week live programme in agentic systems architecture, taught by Sunil Mathew.</t>
         </is>
       </c>
     </row>
     <row r="57" ht="15" customHeight="1">
       <c r="A57" s="10" t="inlineStr">
         <is>
-          <t>6 weeks, live, at ~5 hrs / week. The cohort is capped at 8 seats. Starts October 2026.</t>
+          <t>The Living Craft is a 6-week live programme in agentic systems architecture, taught by Sunil Mathew.</t>
         </is>
       </c>
     </row>
     <row r="58" ht="15" customHeight="1">
       <c r="A58" s="10" t="inlineStr">
         <is>
+          <t>6 weeks, live, at ~5 hrs / week. The cohort is capped at 8 seats. Starts October 2026.</t>
+        </is>
+      </c>
+    </row>
+    <row r="59" ht="15" customHeight="1">
+      <c r="A59" s="10" t="inlineStr">
+        <is>
           <t>By application; every application read personally. Applying commits you to nothing.</t>
         </is>
       </c>
     </row>
-    <row r="59">
-      <c r="A59" s="11" t="inlineStr">
+    <row r="60">
+      <c r="A60" s="11" t="inlineStr">
         <is>
           <t>Apply at https://learning.thelivingcraft.ai/#apply</t>
         </is>
       </c>
     </row>
-    <row r="61" ht="30" customHeight="1">
-      <c r="A61" s="12" t="inlineStr">
+    <row r="62" ht="30" customHeight="1">
+      <c r="A62" s="12" t="inlineStr">
         <is>
           <t>The Run-Cost Model Tool · The Living Craft · Built by Sunil Mathew, co-authored with Claude · free to use and to pass on</t>
         </is>
@@ -930,7 +937,7 @@
     </row>
   </sheetData>
   <hyperlinks>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A59" r:id="rId1"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A60" r:id="rId1"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -1040,12 +1047,12 @@
     <row r="8" ht="26" customHeight="1">
       <c r="D8" s="16" t="inlineStr">
         <is>
-          <t>Plain code. No model.</t>
+          <t>Plain code, from the rules the team already knew.</t>
         </is>
       </c>
       <c r="E8" s="16" t="inlineStr">
         <is>
-          <t>Same code, rebuilt on the written spec.</t>
+          <t>Plain code again, rebuilt on every rule the agent build forced you to write down.</t>
         </is>
       </c>
       <c r="F8" s="16" t="inlineStr">
@@ -2492,12 +2499,12 @@
     <row r="15" ht="26" customHeight="1">
       <c r="D15" s="16" t="inlineStr">
         <is>
-          <t>Plain code. No model.</t>
+          <t>Plain code, from the rules the team already knew.</t>
         </is>
       </c>
       <c r="E15" s="16" t="inlineStr">
         <is>
-          <t>Same code, rebuilt on the written spec.</t>
+          <t>Plain code again, rebuilt on every rule the agent build forced you to write down.</t>
         </is>
       </c>
       <c r="F15" s="16" t="inlineStr">

</xml_diff>